<commit_message>
chore(docs): update economy spreadsheet + skill; ignore tarballs/lockfiles
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="721">
   <si>
     <t xml:space="preserve">Constant</t>
   </si>
@@ -166,7 +166,7 @@
     <t xml:space="preserve">Cardinal Sins, Devotion &amp; Levels</t>
   </si>
   <si>
-    <t xml:space="preserve">Level treshold (total devotion needed) = 180^X (cumulative), where X is level. Skill intensity = (LN(Y)^2)/6.537, where Y is total devotion.</t>
+    <t xml:space="preserve">Level treshold (total devotion needed) = 180^X (cumulative), where X is level. Skill intensity = (LN(Y)^2)/0.6537, where Y is total devotion.</t>
   </si>
   <si>
     <t xml:space="preserve">Prince</t>
@@ -412,7 +412,7 @@
     <t xml:space="preserve">Action efficiency modifies costs and outcomes by the same %; does NOT affect action time.</t>
   </si>
   <si>
-    <t xml:space="preserve">Suggestion  —  one-shot 10s, 5 influence; Luxuria 1 enables toggle</t>
+    <t xml:space="preserve">Suggestion  —  one-shot 5s, 5 influence; Luxuria 1 enables toggle</t>
   </si>
   <si>
     <t xml:space="preserve">Early-game reprobate source.</t>
@@ -1150,7 +1150,7 @@
     <t xml:space="preserve">Indagatio (search) &amp; Emptio (purchase)</t>
   </si>
   <si>
-    <t xml:space="preserve">Action effect reduces action time needed for Indagatio and Emptio (times are in the Globals sheet)</t>
+    <t xml:space="preserve">Action effect reduces action time needed for Indagatio and Emptio</t>
   </si>
   <si>
     <t xml:space="preserve">Indagatio tier</t>
@@ -1159,9 +1159,15 @@
     <t xml:space="preserve">Prob %</t>
   </si>
   <si>
+    <t xml:space="preserve">Indagatio time</t>
+  </si>
+  <si>
     <t xml:space="preserve">Random anathema maleficium found</t>
   </si>
   <si>
+    <t xml:space="preserve">300 s</t>
+  </si>
+  <si>
     <t xml:space="preserve">Random profane maleficium found</t>
   </si>
   <si>
@@ -1183,7 +1189,13 @@
     <t xml:space="preserve">Emptio tier</t>
   </si>
   <si>
+    <t xml:space="preserve">Emptio time</t>
+  </si>
+  <si>
     <t xml:space="preserve">seller vulnerable; kill &amp; take free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 s</t>
   </si>
   <si>
     <t xml:space="preserve">purchase at lower price</t>
@@ -2305,6 +2317,7 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2535,7 +2548,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3146,37 +3159,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>176</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>299</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>299</v>
@@ -3184,13 +3197,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3199,13 +3212,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>58</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="D7" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3214,13 +3227,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3229,13 +3242,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3244,13 +3257,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3259,13 +3272,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>82</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3274,13 +3287,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>88</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3289,13 +3302,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>94</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3333,38 +3346,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="33" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3372,16 +3385,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F5" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3400,16 +3413,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F6" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3428,16 +3441,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>428</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>430</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>424</v>
       </c>
       <c r="F7" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3456,16 +3469,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3484,16 +3497,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F9" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3512,16 +3525,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F10" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3540,16 +3553,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F11" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3568,16 +3581,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F12" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3596,16 +3609,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F13" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3624,16 +3637,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F14" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3652,16 +3665,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F15" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3680,16 +3693,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F16" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3708,16 +3721,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F17" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3736,16 +3749,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F18" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3764,16 +3777,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F19" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3792,16 +3805,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F20" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3820,16 +3833,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F21" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3848,16 +3861,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F22" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3876,16 +3889,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F23" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3904,16 +3917,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F24" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3932,16 +3945,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F25" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3960,16 +3973,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F26" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -3988,16 +4001,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F27" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4016,16 +4029,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F28" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4044,16 +4057,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F29" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4072,16 +4085,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F30" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4100,16 +4113,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F31" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4128,16 +4141,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F32" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4156,16 +4169,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F33" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4184,16 +4197,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F34" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4212,16 +4225,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F35" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4240,16 +4253,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F36" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4268,16 +4281,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F37" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4296,16 +4309,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F38" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4324,16 +4337,16 @@
         <v>35</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F39" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4352,16 +4365,16 @@
         <v>36</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F40" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4380,16 +4393,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F41" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4408,16 +4421,16 @@
         <v>38</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F42" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4436,16 +4449,16 @@
         <v>39</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F43" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4464,16 +4477,16 @@
         <v>40</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F44" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4492,16 +4505,16 @@
         <v>41</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F45" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4520,16 +4533,16 @@
         <v>42</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F46" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4548,16 +4561,16 @@
         <v>43</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F47" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4576,16 +4589,16 @@
         <v>44</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F48" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4604,16 +4617,16 @@
         <v>45</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F49" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4632,16 +4645,16 @@
         <v>46</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F50" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4660,16 +4673,16 @@
         <v>47</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F51" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4688,16 +4701,16 @@
         <v>48</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="F52" s="34" t="n">
         <f aca="false">10*Globals!$B$23</f>
@@ -4716,16 +4729,16 @@
         <v>49</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F53" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4744,16 +4757,16 @@
         <v>50</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F54" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4772,16 +4785,16 @@
         <v>51</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F55" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4800,16 +4813,16 @@
         <v>52</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F56" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4828,16 +4841,16 @@
         <v>53</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F57" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4856,16 +4869,16 @@
         <v>54</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F58" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4884,16 +4897,16 @@
         <v>55</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F59" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4912,16 +4925,16 @@
         <v>56</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F60" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4940,16 +4953,16 @@
         <v>57</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F61" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4968,16 +4981,16 @@
         <v>58</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F62" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -4996,16 +5009,16 @@
         <v>59</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F63" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5024,16 +5037,16 @@
         <v>60</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F64" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5052,16 +5065,16 @@
         <v>61</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F65" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5080,16 +5093,16 @@
         <v>62</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F66" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5108,16 +5121,16 @@
         <v>63</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F67" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5136,16 +5149,16 @@
         <v>64</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F68" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5164,16 +5177,16 @@
         <v>65</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F69" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5192,16 +5205,16 @@
         <v>66</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F70" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5220,16 +5233,16 @@
         <v>67</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F71" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5248,16 +5261,16 @@
         <v>68</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F72" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5276,16 +5289,16 @@
         <v>69</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="F73" s="34" t="n">
         <f aca="false">1*Globals!$B$23</f>
@@ -5304,16 +5317,16 @@
         <v>70</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F74" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5332,16 +5345,16 @@
         <v>71</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F75" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5360,16 +5373,16 @@
         <v>72</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F76" s="34" t="n">
         <f aca="false">0.001*Globals!$B$23</f>
@@ -5414,46 +5427,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>294</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>129</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>2</v>
@@ -5462,7 +5475,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="G5" s="18" t="n">
         <v>0.33</v>
@@ -5470,13 +5483,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>2</v>
@@ -5485,7 +5498,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="G6" s="18" t="n">
         <v>0.33</v>
@@ -5493,13 +5506,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>6</v>
@@ -5508,7 +5521,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="G7" s="18" t="n">
         <v>0.66</v>
@@ -5516,13 +5529,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>1</v>
@@ -5531,19 +5544,19 @@
         <v>1</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="G8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>4</v>
@@ -5552,19 +5565,19 @@
         <v>1</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="G9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
+        <v>662</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>658</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>653</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>654</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>2</v>
@@ -5573,19 +5586,19 @@
         <v>1</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="G10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>8</v>
@@ -5594,19 +5607,19 @@
         <v>1</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="G11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>4</v>
@@ -5615,19 +5628,19 @@
         <v>1</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="G12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>0</v>
@@ -5636,7 +5649,7 @@
         <v>5</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>0.05</v>
@@ -5644,43 +5657,43 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="G14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>1</v>
@@ -5688,13 +5701,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>1</v>
@@ -5703,19 +5716,19 @@
         <v>1</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="G16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>3</v>
@@ -5724,19 +5737,19 @@
         <v>1</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="G17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>1</v>
@@ -5745,40 +5758,40 @@
         <v>1</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="G18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="G19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>0</v>
@@ -5787,7 +5800,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="G20" s="18" t="n">
         <v>3</v>
@@ -5795,13 +5808,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>0</v>
@@ -5810,7 +5823,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="G21" s="18" t="n">
         <v>3</v>
@@ -5818,13 +5831,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>687</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>682</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>683</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>0</v>
@@ -5833,7 +5846,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="G22" s="18" t="n">
         <v>0</v>
@@ -5841,13 +5854,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>0</v>
@@ -5856,7 +5869,7 @@
         <v>1</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="G23" s="18" t="n">
         <v>3</v>
@@ -5864,13 +5877,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>0</v>
@@ -5879,7 +5892,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="G24" s="18" t="n">
         <v>0.5</v>
@@ -5887,22 +5900,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="G25" s="18" t="n">
         <v>0.01</v>
@@ -5910,13 +5923,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>2</v>
@@ -5925,19 +5938,19 @@
         <v>1</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="G26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>1</v>
@@ -5946,19 +5959,19 @@
         <v>1</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="G27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>2</v>
@@ -5967,19 +5980,19 @@
         <v>1</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="G28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>1</v>
@@ -5988,48 +6001,48 @@
         <v>1</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="G29" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
     </row>
   </sheetData>
@@ -6059,26 +6072,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6142,21 +6155,21 @@
         <v>0.33</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>0.33</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
     </row>
   </sheetData>
@@ -6407,7 +6420,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="16" t="n">
-        <f aca="false">(LN(A17)^2)/6.537</f>
+        <f aca="false">(LN(A17)^2)/65.37</f>
         <v>0</v>
       </c>
     </row>
@@ -6416,8 +6429,8 @@
         <v>10</v>
       </c>
       <c r="B18" s="16" t="n">
-        <f aca="false">(LN(A18)^2)/6.537</f>
-        <v>0.811059830270522</v>
+        <f aca="false">(LN(A18)^2)/65.37</f>
+        <v>0.0811059830270521</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6425,8 +6438,8 @@
         <v>50</v>
       </c>
       <c r="B19" s="16" t="n">
-        <f aca="false">(LN(A19)^2)/6.537</f>
-        <v>2.34112345035935</v>
+        <f aca="false">(LN(A19)^2)/65.37</f>
+        <v>0.234112345035935</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6434,8 +6447,8 @@
         <v>180</v>
       </c>
       <c r="B20" s="16" t="n">
-        <f aca="false">(LN(A20)^2)/6.537</f>
-        <v>4.12525636457206</v>
+        <f aca="false">(LN(A20)^2)/65.37</f>
+        <v>0.412525636457206</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6443,8 +6456,8 @@
         <v>1000</v>
       </c>
       <c r="B21" s="16" t="n">
-        <f aca="false">(LN(A21)^2)/6.537</f>
-        <v>7.29953847243469</v>
+        <f aca="false">(LN(A21)^2)/65.37</f>
+        <v>0.729953847243469</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6452,8 +6465,8 @@
         <v>32400</v>
       </c>
       <c r="B22" s="16" t="n">
-        <f aca="false">(LN(A22)^2)/6.537</f>
-        <v>16.5010254582882</v>
+        <f aca="false">(LN(A22)^2)/65.37</f>
+        <v>1.65010254582882</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6461,8 +6474,8 @@
         <v>5832000</v>
       </c>
       <c r="B23" s="16" t="n">
-        <f aca="false">(LN(A23)^2)/6.537</f>
-        <v>37.1273072811486</v>
+        <f aca="false">(LN(A23)^2)/65.37</f>
+        <v>3.71273072811486</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6470,8 +6483,8 @@
         <v>1049760000</v>
       </c>
       <c r="B24" s="16" t="n">
-        <f aca="false">(LN(A24)^2)/6.537</f>
-        <v>66.004101833153</v>
+        <f aca="false">(LN(A24)^2)/65.37</f>
+        <v>6.6004101833153</v>
       </c>
     </row>
   </sheetData>
@@ -6736,7 +6749,7 @@
         <v>112</v>
       </c>
       <c r="B9" s="10" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>132</v>
@@ -6747,7 +6760,7 @@
         <v>114</v>
       </c>
       <c r="B10" s="10" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>133</v>
@@ -6758,7 +6771,7 @@
         <v>116</v>
       </c>
       <c r="B11" s="10" t="n">
-        <v>0.125</v>
+        <v>0.075</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>134</v>
@@ -6839,7 +6852,7 @@
         <v>112</v>
       </c>
       <c r="B20" s="10" t="n">
-        <v>0.525</v>
+        <v>0.575</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>142</v>
@@ -6850,7 +6863,7 @@
         <v>114</v>
       </c>
       <c r="B21" s="10" t="n">
-        <v>0.175</v>
+        <v>0.125</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>133</v>
@@ -7038,7 +7051,7 @@
         <v>112</v>
       </c>
       <c r="B9" s="31" t="n">
-        <v>0.5</v>
+        <v>0.66</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>154</v>
@@ -7049,7 +7062,7 @@
         <v>114</v>
       </c>
       <c r="B10" s="31" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>155</v>
@@ -7060,7 +7073,7 @@
         <v>116</v>
       </c>
       <c r="B11" s="31" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>156</v>
@@ -7071,7 +7084,7 @@
         <v>118</v>
       </c>
       <c r="B12" s="31" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>157</v>
@@ -7152,7 +7165,7 @@
         <v>112</v>
       </c>
       <c r="B21" s="31" t="n">
-        <v>0.5</v>
+        <v>0.66</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>163</v>
@@ -7163,7 +7176,7 @@
         <v>114</v>
       </c>
       <c r="B22" s="31" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>164</v>
@@ -7174,7 +7187,7 @@
         <v>116</v>
       </c>
       <c r="B23" s="31" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>165</v>
@@ -7185,7 +7198,7 @@
         <v>118</v>
       </c>
       <c r="B24" s="31" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>166</v>
@@ -7266,7 +7279,7 @@
         <v>112</v>
       </c>
       <c r="B33" s="31" t="n">
-        <v>0.5</v>
+        <v>0.66</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>172</v>
@@ -7277,7 +7290,7 @@
         <v>114</v>
       </c>
       <c r="B34" s="31" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>164</v>
@@ -7288,7 +7301,7 @@
         <v>116</v>
       </c>
       <c r="B35" s="31" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>165</v>
@@ -7299,7 +7312,7 @@
         <v>118</v>
       </c>
       <c r="B36" s="31" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>166</v>
@@ -7420,7 +7433,7 @@
         <v>185</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>1000</v>
@@ -7429,7 +7442,7 @@
         <v>60</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H5" s="16" t="n">
         <v>1</v>
@@ -7452,16 +7465,16 @@
         <v>187</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H6" s="16" t="n">
         <v>5</v>
@@ -7484,22 +7497,23 @@
         <v>188</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I7" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>186</v>
@@ -7516,22 +7530,22 @@
         <v>189</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H8" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I8" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>186</v>
@@ -7548,7 +7562,7 @@
         <v>190</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>1000</v>
@@ -7557,7 +7571,7 @@
         <v>60</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H9" s="16" t="n">
         <v>1</v>
@@ -7580,16 +7594,16 @@
         <v>192</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H10" s="16" t="n">
         <v>5</v>
@@ -7612,22 +7626,23 @@
         <v>193</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I11" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>191</v>
@@ -7644,22 +7659,22 @@
         <v>194</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H12" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I12" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>191</v>
@@ -7676,7 +7691,7 @@
         <v>195</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>1000</v>
@@ -7685,7 +7700,7 @@
         <v>60</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H13" s="16" t="n">
         <v>1</v>
@@ -7708,16 +7723,16 @@
         <v>197</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H14" s="16" t="n">
         <v>5</v>
@@ -7740,22 +7755,23 @@
         <v>198</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I15" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>196</v>
@@ -7772,22 +7788,22 @@
         <v>199</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H16" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I16" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>196</v>
@@ -7804,7 +7820,7 @@
         <v>200</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>1000</v>
@@ -7813,7 +7829,7 @@
         <v>60</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H17" s="16" t="n">
         <v>1</v>
@@ -7836,16 +7852,16 @@
         <v>202</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G18" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H18" s="16" t="n">
         <v>5</v>
@@ -7868,22 +7884,23 @@
         <v>203</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G19" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I19" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>201</v>
@@ -7900,22 +7917,22 @@
         <v>204</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G20" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H20" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I20" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J20" s="5" t="s">
         <v>201</v>
@@ -7932,7 +7949,7 @@
         <v>205</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>1000</v>
@@ -7941,7 +7958,7 @@
         <v>60</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H21" s="16" t="n">
         <v>1</v>
@@ -7964,16 +7981,16 @@
         <v>207</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G22" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H22" s="16" t="n">
         <v>5</v>
@@ -7996,22 +8013,23 @@
         <v>208</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G23" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I23" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>206</v>
@@ -8028,22 +8046,22 @@
         <v>209</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G24" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H24" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>206</v>
@@ -8060,7 +8078,7 @@
         <v>210</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="5" t="n">
         <v>1000</v>
@@ -8069,7 +8087,7 @@
         <v>60</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H25" s="16" t="n">
         <v>1</v>
@@ -8092,16 +8110,16 @@
         <v>212</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H26" s="16" t="n">
         <v>5</v>
@@ -8124,22 +8142,23 @@
         <v>213</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F27" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H27" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I27" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>211</v>
@@ -8156,22 +8175,22 @@
         <v>214</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G28" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H28" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I28" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>211</v>
@@ -8188,7 +8207,7 @@
         <v>215</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" s="5" t="n">
         <v>1000</v>
@@ -8197,7 +8216,7 @@
         <v>60</v>
       </c>
       <c r="G29" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H29" s="16" t="n">
         <v>1</v>
@@ -8220,16 +8239,16 @@
         <v>217</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F30" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G30" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H30" s="16" t="n">
         <v>5</v>
@@ -8252,22 +8271,23 @@
         <v>218</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G31" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H31" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I31" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>216</v>
@@ -8284,22 +8304,22 @@
         <v>219</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F32" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G32" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H32" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I32" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J32" s="5" t="s">
         <v>216</v>
@@ -8316,7 +8336,7 @@
         <v>220</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" s="5" t="n">
         <v>1000</v>
@@ -8325,7 +8345,7 @@
         <v>60</v>
       </c>
       <c r="G33" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H33" s="16" t="n">
         <v>1</v>
@@ -8348,16 +8368,16 @@
         <v>222</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G34" s="16" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H34" s="16" t="n">
         <v>5</v>
@@ -8380,22 +8400,23 @@
         <v>223</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F35" s="5" t="n">
         <v>36000</v>
       </c>
       <c r="G35" s="16" t="n">
-        <v>750</v>
+        <f aca="false">450</f>
+        <v>450</v>
       </c>
       <c r="H35" s="16" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="I35" s="19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>221</v>
@@ -8412,22 +8433,22 @@
         <v>224</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>1000000000</v>
+        <v>100000000</v>
       </c>
       <c r="F36" s="5" t="n">
         <v>500000</v>
       </c>
       <c r="G36" s="16" t="n">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="H36" s="16" t="n">
         <v>500</v>
       </c>
       <c r="I36" s="19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="J36" s="5" t="s">
         <v>221</v>
@@ -9540,7 +9561,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1048576"/>
+  <dimension ref="A1:D1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -9569,6 +9590,9 @@
       <c r="C4" s="2" t="s">
         <v>129</v>
       </c>
+      <c r="D4" s="2" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
@@ -9578,7 +9602,10 @@
         <v>0.001</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,7 +9616,7 @@
         <v>0.049</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9597,10 +9624,10 @@
         <v>112</v>
       </c>
       <c r="B7" s="10" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9608,10 +9635,10 @@
         <v>114</v>
       </c>
       <c r="B8" s="10" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9622,7 +9649,7 @@
         <v>0.2</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9633,7 +9660,7 @@
         <v>0.045</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9644,7 +9671,7 @@
         <v>0.005</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9659,13 +9686,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>374</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>129</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9676,7 +9706,10 @@
         <v>0.01</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>383</v>
+        <v>386</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9687,7 +9720,7 @@
         <v>0.04</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9698,7 +9731,7 @@
         <v>0.9</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9709,7 +9742,7 @@
         <v>0.049</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9720,7 +9753,7 @@
         <v>0.001</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Phase 4: delegation engine, invocations, Katabasis freeze, success shifts
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -2852,7 +2852,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>5</v>
@@ -7445,7 +7445,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="16" t="n">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="I5" s="19" t="n">
         <v>0.01</v>
@@ -7477,7 +7477,7 @@
         <v>22</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I6" s="19" t="n">
         <v>0.025</v>

</xml_diff>

<commit_message>
feat(web): uniform degradation pass over room scenes + prop-driven Ars Goetia rework
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -7535,7 +7535,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>60</v>
@@ -7664,7 +7664,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>60</v>
@@ -7793,7 +7793,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>60</v>
@@ -7922,7 +7922,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>60</v>
@@ -8051,7 +8051,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>60</v>
@@ -8180,7 +8180,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>60</v>
@@ -8309,7 +8309,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F33" s="5" t="n">
         <v>60</v>

</xml_diff>

<commit_message>
refactor(web): decouple Ars Goetia types from the degradation layer (no visual change)
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="717">
   <si>
     <t xml:space="preserve">Constant</t>
   </si>
@@ -2175,9 +2175,6 @@
   </si>
   <si>
     <t xml:space="preserve">Note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 = visual cap in Altar room</t>
   </si>
   <si>
     <t xml:space="preserve">L* 2.2</t>
@@ -6066,21 +6063,19 @@
         <v>110</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>0.33</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>299</v>
-      </c>
+      <c r="D5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
         <v>242</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>0.33</v>
@@ -6093,7 +6088,7 @@
         <v>532.4</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>0.33</v>
@@ -6106,41 +6101,32 @@
         <v>1170.4</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>0.33</v>
       </c>
       <c r="D8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
-        <f aca="false">1170*2.2</f>
-        <v>2574</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>4</v>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>714</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>715</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>0.33</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>714</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>715</v>
-      </c>
-      <c r="B10" s="5" t="s">
         <v>716</v>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>717</v>
-      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0"/>
+      <c r="B10" s="0"/>
+      <c r="C10" s="0"/>
+      <c r="D10" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
content(web): Familiar without numeral, drop turn-the-leaf, rewrite Ars Goetia intro
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="727">
   <si>
     <t xml:space="preserve">Constant</t>
   </si>
@@ -919,6 +919,12 @@
     <t xml:space="preserve">Efficiency (compared to player base efficiency)</t>
   </si>
   <si>
+    <t xml:space="preserve">Visually displayed once invoked?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle movement?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Familiar</t>
   </si>
   <si>
@@ -937,6 +943,12 @@
     <t xml:space="preserve">Flat +33% player eff; Action efficiency applies to Indagatio.</t>
   </si>
   <si>
+    <t xml:space="preserve">Always in the Studio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve">Upir</t>
   </si>
   <si>
@@ -952,6 +964,9 @@
     <t xml:space="preserve">Action efficiency applies to Caedis</t>
   </si>
   <si>
+    <t xml:space="preserve">10% times in the invocation room</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aurevora</t>
   </si>
   <si>
@@ -970,6 +985,10 @@
     <t xml:space="preserve">-%</t>
   </si>
   <si>
+    <t xml:space="preserve">Immediately when invoked, overrides other invocations in the room.
+Only disappears when dispelled.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lamia</t>
   </si>
   <si>
@@ -985,6 +1004,9 @@
     <t xml:space="preserve">Action efficiency applies to Suasio</t>
   </si>
   <si>
+    <t xml:space="preserve">Immediately when invoked.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Succubus</t>
   </si>
   <si>
@@ -1006,6 +1028,9 @@
     <t xml:space="preserve">Action efficiency applies as increase to Vitium Mercatura output</t>
   </si>
   <si>
+    <t xml:space="preserve">10% times in the Studio.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Midas</t>
   </si>
   <si>
@@ -1097,6 +1122,12 @@
   </si>
   <si>
     <t xml:space="preserve">full freeze; next Katabasis 100% gold/maleficia, keep Emptio list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floating over the Altar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
   </si>
   <si>
     <t xml:space="preserve">Fama</t>
@@ -2199,7 +2230,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.00"/>
     <numFmt numFmtId="170" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2306,6 +2337,12 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2419,7 +2456,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2550,6 +2587,14 @@
     </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -3123,51 +3168,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>173</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3176,13 +3221,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>398</v>
+        <v>408</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>55</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
       <c r="D7" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3191,13 +3236,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>61</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>401</v>
+        <v>411</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3206,13 +3251,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>402</v>
+        <v>412</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>67</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3221,13 +3266,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>73</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3236,13 +3281,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>406</v>
+        <v>416</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>79</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>407</v>
+        <v>417</v>
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3251,13 +3296,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>85</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3266,13 +3311,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">Globals!$B$5</f>
@@ -3310,38 +3355,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="33" t="s">
-        <v>413</v>
+      <c r="A2" s="35" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3349,18 +3394,18 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F5" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F5" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3377,18 +3422,18 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F6" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F6" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3405,18 +3450,18 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F7" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F7" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3433,18 +3478,18 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>432</v>
+        <v>442</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>433</v>
+        <v>443</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>434</v>
+        <v>444</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F8" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F8" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3461,18 +3506,18 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3489,18 +3534,18 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F10" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F10" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3517,18 +3562,18 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>441</v>
+        <v>451</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F11" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F11" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3545,18 +3590,18 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F12" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F12" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3573,18 +3618,18 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F13" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F13" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3601,18 +3646,18 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F14" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F14" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3629,18 +3674,18 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F15" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F15" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3657,18 +3702,18 @@
         <v>12</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>456</v>
+        <v>466</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F16" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F16" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3685,18 +3730,18 @@
         <v>13</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F17" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F17" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3713,18 +3758,18 @@
         <v>14</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>463</v>
+        <v>473</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F18" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F18" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3741,18 +3786,18 @@
         <v>15</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F19" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F19" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3769,18 +3814,18 @@
         <v>16</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>468</v>
+        <v>478</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>469</v>
+        <v>479</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F20" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F20" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3797,18 +3842,18 @@
         <v>17</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>472</v>
+        <v>482</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>473</v>
+        <v>483</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F21" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F21" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3825,18 +3870,18 @@
         <v>18</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>475</v>
+        <v>485</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F22" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F22" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3853,18 +3898,18 @@
         <v>19</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F23" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F23" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3881,18 +3926,18 @@
         <v>20</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F24" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F24" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3909,18 +3954,18 @@
         <v>21</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F25" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F25" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3937,18 +3982,18 @@
         <v>22</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>486</v>
+        <v>496</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F26" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F26" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3965,18 +4010,18 @@
         <v>23</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>489</v>
+        <v>499</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>491</v>
+        <v>501</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F27" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F27" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3993,18 +4038,18 @@
         <v>24</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>492</v>
+        <v>502</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F28" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F28" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4021,18 +4066,18 @@
         <v>25</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F29" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F29" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4049,18 +4094,18 @@
         <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>500</v>
+        <v>510</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F30" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F30" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4077,18 +4122,18 @@
         <v>27</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>502</v>
+        <v>512</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F31" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F31" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4105,18 +4150,18 @@
         <v>28</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>506</v>
+        <v>516</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F32" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F32" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4133,18 +4178,18 @@
         <v>29</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>507</v>
+        <v>517</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>508</v>
+        <v>518</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>509</v>
+        <v>519</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F33" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F33" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4161,18 +4206,18 @@
         <v>30</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>511</v>
+        <v>521</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>512</v>
+        <v>522</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F34" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F34" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4189,18 +4234,18 @@
         <v>31</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>513</v>
+        <v>523</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>514</v>
+        <v>524</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>515</v>
+        <v>525</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F35" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F35" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4217,18 +4262,18 @@
         <v>32</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>516</v>
+        <v>526</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>517</v>
+        <v>527</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>518</v>
+        <v>528</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F36" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F36" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4245,18 +4290,18 @@
         <v>33</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>521</v>
+        <v>531</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F37" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F37" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4273,18 +4318,18 @@
         <v>34</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>523</v>
+        <v>533</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>524</v>
+        <v>534</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F38" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F38" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4301,18 +4346,18 @@
         <v>35</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>525</v>
+        <v>535</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>526</v>
+        <v>536</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F39" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F39" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4329,18 +4374,18 @@
         <v>36</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>528</v>
+        <v>538</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F40" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F40" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4357,18 +4402,18 @@
         <v>37</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F41" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F41" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4385,18 +4430,18 @@
         <v>38</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F42" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F42" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4413,18 +4458,18 @@
         <v>39</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>536</v>
+        <v>546</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>538</v>
+        <v>548</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F43" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F43" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4441,18 +4486,18 @@
         <v>40</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>539</v>
+        <v>549</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F44" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F44" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4469,18 +4514,18 @@
         <v>41</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>542</v>
+        <v>552</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>543</v>
+        <v>553</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F45" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F45" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4497,18 +4542,18 @@
         <v>42</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>546</v>
+        <v>556</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F46" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F46" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4525,18 +4570,18 @@
         <v>43</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>549</v>
+        <v>559</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F47" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F47" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4553,18 +4598,18 @@
         <v>44</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>551</v>
+        <v>561</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>552</v>
+        <v>562</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F48" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F48" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4581,18 +4626,18 @@
         <v>45</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>553</v>
+        <v>563</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F49" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F49" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4609,18 +4654,18 @@
         <v>46</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>556</v>
+        <v>566</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>557</v>
+        <v>567</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>558</v>
+        <v>568</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F50" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F50" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4637,18 +4682,18 @@
         <v>47</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>559</v>
+        <v>569</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F51" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F51" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4665,18 +4710,18 @@
         <v>48</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>562</v>
+        <v>572</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>563</v>
+        <v>573</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>564</v>
+        <v>574</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>565</v>
-      </c>
-      <c r="F52" s="34" t="n">
+        <v>575</v>
+      </c>
+      <c r="F52" s="36" t="n">
         <f aca="false">10*Globals!$B$21</f>
         <v>10</v>
       </c>
@@ -4693,18 +4738,18 @@
         <v>49</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>566</v>
+        <v>576</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>567</v>
+        <v>577</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>568</v>
+        <v>578</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F53" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F53" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4721,18 +4766,18 @@
         <v>50</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>569</v>
+        <v>579</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F54" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F54" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4749,18 +4794,18 @@
         <v>51</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>572</v>
+        <v>582</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>573</v>
+        <v>583</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>574</v>
+        <v>584</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F55" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F55" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4777,18 +4822,18 @@
         <v>52</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>575</v>
+        <v>585</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>576</v>
+        <v>586</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>577</v>
+        <v>587</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F56" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F56" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4805,18 +4850,18 @@
         <v>53</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>578</v>
+        <v>588</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>579</v>
+        <v>589</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>580</v>
+        <v>590</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F57" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F57" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4833,18 +4878,18 @@
         <v>54</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>581</v>
+        <v>591</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>583</v>
+        <v>593</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F58" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F58" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4861,18 +4906,18 @@
         <v>55</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>584</v>
+        <v>594</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>585</v>
+        <v>595</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>586</v>
+        <v>596</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F59" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F59" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4889,18 +4934,18 @@
         <v>56</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>587</v>
+        <v>597</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>588</v>
+        <v>598</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>589</v>
+        <v>599</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F60" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F60" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4917,18 +4962,18 @@
         <v>57</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>590</v>
+        <v>600</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>591</v>
+        <v>601</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>592</v>
+        <v>602</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F61" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F61" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4945,18 +4990,18 @@
         <v>58</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>593</v>
+        <v>603</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>594</v>
+        <v>604</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>595</v>
+        <v>605</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F62" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F62" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4973,18 +5018,18 @@
         <v>59</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>596</v>
+        <v>606</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>597</v>
+        <v>607</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>598</v>
+        <v>608</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F63" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F63" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5001,18 +5046,18 @@
         <v>60</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>599</v>
+        <v>609</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>600</v>
+        <v>610</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>601</v>
+        <v>611</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F64" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F64" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5029,18 +5074,18 @@
         <v>61</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>602</v>
+        <v>612</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>603</v>
+        <v>613</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>604</v>
+        <v>614</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F65" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F65" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5057,18 +5102,18 @@
         <v>62</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>605</v>
+        <v>615</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>606</v>
+        <v>616</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>607</v>
+        <v>617</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F66" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F66" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5085,18 +5130,18 @@
         <v>63</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>608</v>
+        <v>618</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>609</v>
+        <v>619</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>610</v>
+        <v>620</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F67" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F67" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5113,18 +5158,18 @@
         <v>64</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>611</v>
+        <v>621</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>612</v>
+        <v>622</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>613</v>
+        <v>623</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F68" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F68" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5141,18 +5186,18 @@
         <v>65</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>614</v>
+        <v>624</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>615</v>
+        <v>625</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>616</v>
+        <v>626</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F69" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F69" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5169,18 +5214,18 @@
         <v>66</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>617</v>
+        <v>627</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>618</v>
+        <v>628</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F70" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F70" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5197,18 +5242,18 @@
         <v>67</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>619</v>
+        <v>629</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>620</v>
+        <v>630</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>621</v>
+        <v>631</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F71" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F71" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5225,18 +5270,18 @@
         <v>68</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>622</v>
+        <v>632</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>623</v>
+        <v>633</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>624</v>
+        <v>634</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F72" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F72" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5253,18 +5298,18 @@
         <v>69</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>625</v>
+        <v>635</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>626</v>
+        <v>636</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>627</v>
+        <v>637</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>565</v>
-      </c>
-      <c r="F73" s="34" t="n">
+        <v>575</v>
+      </c>
+      <c r="F73" s="36" t="n">
         <f aca="false">1*Globals!$B$21</f>
         <v>1</v>
       </c>
@@ -5281,18 +5326,18 @@
         <v>70</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>628</v>
+        <v>638</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>629</v>
+        <v>639</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>630</v>
+        <v>640</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F74" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F74" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5309,18 +5354,18 @@
         <v>71</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>631</v>
+        <v>641</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>632</v>
+        <v>642</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>633</v>
+        <v>643</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F75" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F75" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5337,18 +5382,18 @@
         <v>72</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>634</v>
+        <v>644</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>635</v>
+        <v>645</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>636</v>
+        <v>646</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="F76" s="34" t="n">
+        <v>435</v>
+      </c>
+      <c r="F76" s="36" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5391,46 +5436,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>637</v>
+        <v>647</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>638</v>
+        <v>648</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>291</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>640</v>
+        <v>650</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>641</v>
+        <v>651</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>642</v>
+        <v>652</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>126</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>643</v>
+        <v>653</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>644</v>
+        <v>654</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>645</v>
+        <v>655</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>2</v>
@@ -5439,7 +5484,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>647</v>
+        <v>657</v>
       </c>
       <c r="G5" s="18" t="n">
         <v>0.33</v>
@@ -5447,13 +5492,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>648</v>
+        <v>658</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>645</v>
+        <v>655</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>2</v>
@@ -5462,7 +5507,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>649</v>
+        <v>659</v>
       </c>
       <c r="G6" s="18" t="n">
         <v>0.33</v>
@@ -5470,13 +5515,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>650</v>
+        <v>660</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>645</v>
+        <v>655</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>651</v>
+        <v>661</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>6</v>
@@ -5485,7 +5530,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>652</v>
+        <v>662</v>
       </c>
       <c r="G7" s="18" t="n">
         <v>0.66</v>
@@ -5493,13 +5538,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>653</v>
+        <v>663</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>1</v>
@@ -5508,19 +5553,19 @@
         <v>1</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>656</v>
+        <v>666</v>
       </c>
       <c r="G8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>657</v>
+        <v>667</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>4</v>
@@ -5529,19 +5574,19 @@
         <v>1</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>658</v>
+        <v>668</v>
       </c>
       <c r="G9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>659</v>
+        <v>669</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>2</v>
@@ -5550,19 +5595,19 @@
         <v>1</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>660</v>
+        <v>670</v>
       </c>
       <c r="G10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
+        <v>671</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>661</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>662</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>651</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>8</v>
@@ -5571,19 +5616,19 @@
         <v>1</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>663</v>
+        <v>673</v>
       </c>
       <c r="G11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
+        <v>674</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>664</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>654</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>4</v>
@@ -5592,19 +5637,19 @@
         <v>1</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>658</v>
+        <v>668</v>
       </c>
       <c r="G12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
+        <v>675</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>676</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>665</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>666</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>655</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>0</v>
@@ -5613,7 +5658,7 @@
         <v>5</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>667</v>
+        <v>677</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>0.05</v>
@@ -5621,43 +5666,43 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>668</v>
+        <v>678</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>651</v>
+        <v>661</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>671</v>
+        <v>681</v>
       </c>
       <c r="G14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>672</v>
+        <v>682</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>673</v>
+        <v>683</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>1</v>
@@ -5665,13 +5710,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>1</v>
@@ -5680,19 +5725,19 @@
         <v>1</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>675</v>
+        <v>685</v>
       </c>
       <c r="G16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>676</v>
+        <v>686</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>3</v>
@@ -5701,19 +5746,19 @@
         <v>1</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="G17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>678</v>
+        <v>688</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>1</v>
@@ -5722,40 +5767,40 @@
         <v>1</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>679</v>
+        <v>689</v>
       </c>
       <c r="G18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>680</v>
+        <v>690</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>656</v>
+        <v>666</v>
       </c>
       <c r="G19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>682</v>
+        <v>692</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>0</v>
@@ -5764,7 +5809,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>685</v>
+        <v>695</v>
       </c>
       <c r="G20" s="18" t="n">
         <v>3</v>
@@ -5772,13 +5817,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>0</v>
@@ -5787,7 +5832,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>687</v>
+        <v>697</v>
       </c>
       <c r="G21" s="18" t="n">
         <v>3</v>
@@ -5795,13 +5840,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>688</v>
+        <v>698</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>0</v>
@@ -5810,7 +5855,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>689</v>
+        <v>699</v>
       </c>
       <c r="G22" s="18" t="n">
         <v>0</v>
@@ -5818,13 +5863,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>690</v>
+        <v>700</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>0</v>
@@ -5833,7 +5878,7 @@
         <v>1</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="G23" s="18" t="n">
         <v>3</v>
@@ -5841,13 +5886,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>692</v>
+        <v>702</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>0</v>
@@ -5856,7 +5901,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>693</v>
+        <v>703</v>
       </c>
       <c r="G24" s="18" t="n">
         <v>0.5</v>
@@ -5864,22 +5909,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>695</v>
+        <v>705</v>
       </c>
       <c r="G25" s="18" t="n">
         <v>0.01</v>
@@ -5887,13 +5932,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>2</v>
@@ -5902,19 +5947,19 @@
         <v>1</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>660</v>
+        <v>670</v>
       </c>
       <c r="G26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>1</v>
@@ -5923,19 +5968,19 @@
         <v>1</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="G27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>2</v>
@@ -5944,19 +5989,19 @@
         <v>1</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>660</v>
+        <v>670</v>
       </c>
       <c r="G28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>1</v>
@@ -5965,48 +6010,48 @@
         <v>1</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>701</v>
+        <v>711</v>
       </c>
       <c r="G29" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>703</v>
+        <v>713</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>651</v>
+        <v>661</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>705</v>
+        <v>715</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
     </row>
   </sheetData>
@@ -6036,26 +6081,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>709</v>
+        <v>719</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>711</v>
+        <v>721</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6110,16 +6155,16 @@
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>0.33</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8971,7 +9016,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -8982,6 +9027,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="57.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -8995,7 +9042,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>287</v>
       </c>
@@ -9020,485 +9067,579 @@
       <c r="H4" s="2" t="s">
         <v>294</v>
       </c>
+      <c r="I4" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H5" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I5" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="J5" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="H6" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I6" s="31" t="s">
+        <v>310</v>
+      </c>
+      <c r="J6" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>311</v>
+        <v>316</v>
+      </c>
+      <c r="I7" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="J7" s="31" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>55</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="H8" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I8" s="34" t="s">
+        <v>323</v>
+      </c>
+      <c r="J8" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>55</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="H9" s="19" t="n">
         <f aca="false">19.8*Globals!$B$9</f>
         <v>0.99</v>
       </c>
+      <c r="I9" s="19" t="s">
+        <v>310</v>
+      </c>
+      <c r="J9" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>61</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="H10" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I10" s="31" t="s">
+        <v>331</v>
+      </c>
+      <c r="J10" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>61</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="H11" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I11" s="31" t="s">
+        <v>331</v>
+      </c>
+      <c r="J11" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>73</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="H12" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>73</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="H13" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>73</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>311</v>
+        <v>316</v>
+      </c>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>67</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="H15" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>67</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="H16" s="31" t="s">
-        <v>311</v>
+        <v>316</v>
+      </c>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>79</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="H17" s="31" t="n">
         <f aca="false">0.5*Globals!$B$9</f>
         <v>0.025</v>
       </c>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>79</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>311</v>
+        <v>316</v>
+      </c>
+      <c r="I18" s="31" t="s">
+        <v>363</v>
+      </c>
+      <c r="J18" s="31" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>85</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
       <c r="H19" s="31" t="n">
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>85</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>311</v>
+        <v>316</v>
+      </c>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="H21" s="31" t="n">
         <f aca="false">0.01*Globals!$B$9</f>
         <v>0.0005</v>
       </c>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>311</v>
+        <v>316</v>
+      </c>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31" t="s">
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -9528,26 +9669,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>126</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9558,10 +9699,10 @@
         <v>0.001</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9572,7 +9713,7 @@
         <v>0.049</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9583,7 +9724,7 @@
         <v>0.2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9594,7 +9735,7 @@
         <v>0.5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9605,7 +9746,7 @@
         <v>0.2</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9616,7 +9757,7 @@
         <v>0.045</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9627,7 +9768,7 @@
         <v>0.005</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9642,16 +9783,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>381</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>371</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>126</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9662,10 +9803,10 @@
         <v>0.01</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9676,7 +9817,7 @@
         <v>0.04</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9687,7 +9828,7 @@
         <v>0.9</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9698,7 +9839,7 @@
         <v>0.049</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9709,7 +9850,7 @@
         <v>0.001</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: consolidate pending UI topics for Claude Design in README
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -502,7 +502,7 @@
     <t xml:space="preserve">Higher power stops the assassination and campaings against you – 66% gold loss and 50% total reprobate loss.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pogrom  —  one-shot ~60s, high gold; unlock Ira 2, toggle Ira 3</t>
+    <t xml:space="preserve">Pogrom  —  one-shot ~60s, 1000 gold; unlock Ira 2, toggle Ira 3</t>
   </si>
   <si>
     <t xml:space="preserve">Single-subtype mass cull (% of chosen subtype).</t>
@@ -529,7 +529,7 @@
     <t xml:space="preserve">Higher power smites your operation – lose 65% of all gold</t>
   </si>
   <si>
-    <t xml:space="preserve">Purgatio  —  one-shot ~3600s, very high gold; unlock Ira 3, toggle Ira 4</t>
+    <t xml:space="preserve">Purgatio  —  one-shot ~3600s, 10000; unlock Ira 3, toggle Ira 4</t>
   </si>
   <si>
     <t xml:space="preserve">All subtypes culled simultaneously. Soul farming.</t>

</xml_diff>

<commit_message>
feat(web): uncap offline progression, bound Acedia compound (ADR-004 amended)
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -2230,7 +2230,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.00"/>
     <numFmt numFmtId="170" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2337,12 +2337,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2456,7 +2450,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2591,10 +2585,6 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -3359,7 +3349,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="34" t="s">
         <v>423</v>
       </c>
     </row>
@@ -3405,7 +3395,7 @@
       <c r="E5" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F5" s="36" t="n">
+      <c r="F5" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3433,7 +3423,7 @@
       <c r="E6" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F6" s="36" t="n">
+      <c r="F6" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3461,7 +3451,7 @@
       <c r="E7" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F7" s="36" t="n">
+      <c r="F7" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3489,7 +3479,7 @@
       <c r="E8" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F8" s="36" t="n">
+      <c r="F8" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3517,7 +3507,7 @@
       <c r="E9" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F9" s="36" t="n">
+      <c r="F9" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3545,7 +3535,7 @@
       <c r="E10" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F10" s="36" t="n">
+      <c r="F10" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3573,7 +3563,7 @@
       <c r="E11" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F11" s="36" t="n">
+      <c r="F11" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3601,7 +3591,7 @@
       <c r="E12" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F12" s="36" t="n">
+      <c r="F12" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3629,7 +3619,7 @@
       <c r="E13" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F13" s="36" t="n">
+      <c r="F13" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3657,7 +3647,7 @@
       <c r="E14" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F14" s="36" t="n">
+      <c r="F14" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3685,7 +3675,7 @@
       <c r="E15" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F15" s="36" t="n">
+      <c r="F15" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3713,7 +3703,7 @@
       <c r="E16" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F16" s="36" t="n">
+      <c r="F16" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3741,7 +3731,7 @@
       <c r="E17" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F17" s="36" t="n">
+      <c r="F17" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3769,7 +3759,7 @@
       <c r="E18" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F18" s="36" t="n">
+      <c r="F18" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3797,7 +3787,7 @@
       <c r="E19" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F19" s="36" t="n">
+      <c r="F19" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3825,7 +3815,7 @@
       <c r="E20" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F20" s="36" t="n">
+      <c r="F20" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3853,7 +3843,7 @@
       <c r="E21" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F21" s="36" t="n">
+      <c r="F21" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3881,7 +3871,7 @@
       <c r="E22" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F22" s="36" t="n">
+      <c r="F22" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3909,7 +3899,7 @@
       <c r="E23" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F23" s="36" t="n">
+      <c r="F23" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3937,7 +3927,7 @@
       <c r="E24" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F24" s="36" t="n">
+      <c r="F24" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3965,7 +3955,7 @@
       <c r="E25" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F25" s="36" t="n">
+      <c r="F25" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -3993,7 +3983,7 @@
       <c r="E26" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F26" s="36" t="n">
+      <c r="F26" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4021,7 +4011,7 @@
       <c r="E27" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F27" s="36" t="n">
+      <c r="F27" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4049,7 +4039,7 @@
       <c r="E28" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F28" s="36" t="n">
+      <c r="F28" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4077,7 +4067,7 @@
       <c r="E29" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F29" s="36" t="n">
+      <c r="F29" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4105,7 +4095,7 @@
       <c r="E30" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F30" s="36" t="n">
+      <c r="F30" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4133,7 +4123,7 @@
       <c r="E31" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F31" s="36" t="n">
+      <c r="F31" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4161,7 +4151,7 @@
       <c r="E32" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F32" s="36" t="n">
+      <c r="F32" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4189,7 +4179,7 @@
       <c r="E33" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F33" s="36" t="n">
+      <c r="F33" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4217,7 +4207,7 @@
       <c r="E34" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F34" s="36" t="n">
+      <c r="F34" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4245,7 +4235,7 @@
       <c r="E35" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F35" s="36" t="n">
+      <c r="F35" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4273,7 +4263,7 @@
       <c r="E36" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F36" s="36" t="n">
+      <c r="F36" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4301,7 +4291,7 @@
       <c r="E37" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F37" s="36" t="n">
+      <c r="F37" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4329,7 +4319,7 @@
       <c r="E38" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F38" s="36" t="n">
+      <c r="F38" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4357,7 +4347,7 @@
       <c r="E39" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F39" s="36" t="n">
+      <c r="F39" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4385,7 +4375,7 @@
       <c r="E40" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F40" s="36" t="n">
+      <c r="F40" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4413,7 +4403,7 @@
       <c r="E41" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F41" s="36" t="n">
+      <c r="F41" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4441,7 +4431,7 @@
       <c r="E42" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F42" s="36" t="n">
+      <c r="F42" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4469,7 +4459,7 @@
       <c r="E43" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F43" s="36" t="n">
+      <c r="F43" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4497,7 +4487,7 @@
       <c r="E44" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F44" s="36" t="n">
+      <c r="F44" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4525,7 +4515,7 @@
       <c r="E45" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F45" s="36" t="n">
+      <c r="F45" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4553,7 +4543,7 @@
       <c r="E46" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F46" s="36" t="n">
+      <c r="F46" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4581,7 +4571,7 @@
       <c r="E47" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F47" s="36" t="n">
+      <c r="F47" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4609,7 +4599,7 @@
       <c r="E48" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F48" s="36" t="n">
+      <c r="F48" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4637,7 +4627,7 @@
       <c r="E49" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F49" s="36" t="n">
+      <c r="F49" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4665,7 +4655,7 @@
       <c r="E50" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F50" s="36" t="n">
+      <c r="F50" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4693,7 +4683,7 @@
       <c r="E51" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F51" s="36" t="n">
+      <c r="F51" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4721,7 +4711,7 @@
       <c r="E52" s="9" t="s">
         <v>575</v>
       </c>
-      <c r="F52" s="36" t="n">
+      <c r="F52" s="35" t="n">
         <f aca="false">10*Globals!$B$21</f>
         <v>10</v>
       </c>
@@ -4749,7 +4739,7 @@
       <c r="E53" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F53" s="36" t="n">
+      <c r="F53" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4777,7 +4767,7 @@
       <c r="E54" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F54" s="36" t="n">
+      <c r="F54" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4805,7 +4795,7 @@
       <c r="E55" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F55" s="36" t="n">
+      <c r="F55" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4833,7 +4823,7 @@
       <c r="E56" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F56" s="36" t="n">
+      <c r="F56" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4861,7 +4851,7 @@
       <c r="E57" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F57" s="36" t="n">
+      <c r="F57" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4889,7 +4879,7 @@
       <c r="E58" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F58" s="36" t="n">
+      <c r="F58" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4917,7 +4907,7 @@
       <c r="E59" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F59" s="36" t="n">
+      <c r="F59" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4945,7 +4935,7 @@
       <c r="E60" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F60" s="36" t="n">
+      <c r="F60" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -4973,7 +4963,7 @@
       <c r="E61" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F61" s="36" t="n">
+      <c r="F61" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5001,7 +4991,7 @@
       <c r="E62" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F62" s="36" t="n">
+      <c r="F62" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5029,7 +5019,7 @@
       <c r="E63" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F63" s="36" t="n">
+      <c r="F63" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5057,7 +5047,7 @@
       <c r="E64" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F64" s="36" t="n">
+      <c r="F64" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5085,7 +5075,7 @@
       <c r="E65" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F65" s="36" t="n">
+      <c r="F65" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5113,7 +5103,7 @@
       <c r="E66" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F66" s="36" t="n">
+      <c r="F66" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5141,7 +5131,7 @@
       <c r="E67" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F67" s="36" t="n">
+      <c r="F67" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5169,7 +5159,7 @@
       <c r="E68" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F68" s="36" t="n">
+      <c r="F68" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5197,7 +5187,7 @@
       <c r="E69" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F69" s="36" t="n">
+      <c r="F69" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5225,7 +5215,7 @@
       <c r="E70" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F70" s="36" t="n">
+      <c r="F70" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5253,7 +5243,7 @@
       <c r="E71" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F71" s="36" t="n">
+      <c r="F71" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5281,7 +5271,7 @@
       <c r="E72" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F72" s="36" t="n">
+      <c r="F72" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5309,7 +5299,7 @@
       <c r="E73" s="9" t="s">
         <v>575</v>
       </c>
-      <c r="F73" s="36" t="n">
+      <c r="F73" s="35" t="n">
         <f aca="false">1*Globals!$B$21</f>
         <v>1</v>
       </c>
@@ -5337,7 +5327,7 @@
       <c r="E74" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F74" s="36" t="n">
+      <c r="F74" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5365,7 +5355,7 @@
       <c r="E75" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F75" s="36" t="n">
+      <c r="F75" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -5393,7 +5383,7 @@
       <c r="E76" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F76" s="36" t="n">
+      <c r="F76" s="35" t="n">
         <f aca="false">0.001*Globals!$B$21</f>
         <v>0.001</v>
       </c>
@@ -6070,7 +6060,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
@@ -6166,12 +6156,6 @@
       <c r="D9" s="6" t="s">
         <v>726</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0"/>
-      <c r="B10" s="0"/>
-      <c r="C10" s="0"/>
-      <c r="D10" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -9027,8 +9011,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="57.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="57.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -9042,7 +9026,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>287</v>
       </c>
@@ -9198,7 +9182,7 @@
         <f aca="false">1*Globals!$B$9</f>
         <v>0.05</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="I8" s="31" t="s">
         <v>323</v>
       </c>
       <c r="J8" s="31" t="s">

</xml_diff>

<commit_message>
feat(sim): Cholerics killable by default; wire Haures #64 (Choleric murder-bias); Imperium 10s
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -457,7 +457,7 @@
     <t xml:space="preserve">reject + redeem -&gt; -1 reprobate</t>
   </si>
   <si>
-    <t xml:space="preserve">Imperium  —  one-shot, 100 influence; unlock Luxuria 3, toggle Luxuria 4</t>
+    <t xml:space="preserve">Imperium  —  one-shot 10s, 100 influence; unlock Luxuria 3, toggle Luxuria 4</t>
   </si>
   <si>
     <t xml:space="preserve">Late-game; outcome is fixed (player in control).</t>
@@ -1749,7 +1749,7 @@
     <t xml:space="preserve">Love of women; all times</t>
   </si>
   <si>
-    <t xml:space="preserve">-Degenerate gold penalty</t>
+    <t xml:space="preserve">-Degenerate suicide and murder rates penalty</t>
   </si>
   <si>
     <t xml:space="preserve">Haagenti</t>

</xml_diff>

<commit_message>
Katabasis backdrops: pixelate + degrade treatment, no palette tint
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId3"/>
@@ -1112,13 +1112,13 @@
     <t xml:space="preserve">gold spent, no outcome</t>
   </si>
   <si>
-    <t xml:space="preserve">5% current gold loss.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15% current gold loss.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">66% gold loss and 50% total reprobate loss.</t>
+    <t xml:space="preserve">5% gold loss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15% gold loss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33% gold loss and 25% total reprobate loss.</t>
   </si>
   <si>
     <t xml:space="preserve">Pogrom  —  one-shot ~60s, 1000 gold; unlock Ira 2, toggle Ira 3</t>
@@ -1136,25 +1136,25 @@
     <t xml:space="preserve">0.1% reprobates die (+= souls)</t>
   </si>
   <si>
-    <t xml:space="preserve">5% current gold loss</t>
+    <t xml:space="preserve">5% gold loss</t>
   </si>
   <si>
     <t xml:space="preserve">Lose 15% reprobates</t>
   </si>
   <si>
+    <t xml:space="preserve">66% gold loss and 50% reprobate loss.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Purgatio  —  one-shot ~360s, 1000000; unlock Ira 3, toggle Ira 4</t>
   </si>
   <si>
     <t xml:space="preserve">Soul farming.</t>
   </si>
   <si>
-    <t xml:space="preserve">25% of all reprobates die (+= souls)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10% of all reprobates die (+= souls)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1% of all reprobates die (+= souls)</t>
+    <t xml:space="preserve">25% reprobates die (+= souls)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10% reprobates die (+= souls)</t>
   </si>
   <si>
     <t xml:space="preserve">Lose 100% gold</t>
@@ -1235,7 +1235,7 @@
     <t xml:space="preserve">Invocatio — Summoning</t>
   </si>
   <si>
-    <t xml:space="preserve">Persistent unless noted; all dispelled on Katabasis. You can only have one Apex invocation active. You can only have one Familiar invocation active. You can have any number of normal invocations active.</t>
+    <t xml:space="preserve">Persistent unless noted; all dispelled on Katabasis. You can only have one Apex invocation active. You can only have one Familiar invocation active. You can have any number of normal invocations active. All invocations visually disappear when dispelled.</t>
   </si>
   <si>
     <t xml:space="preserve">Invocation</t>
@@ -1328,14 +1328,13 @@
     <t xml:space="preserve">(1% * e^s) gold/s</t>
   </si>
   <si>
-    <t xml:space="preserve">Eats 1% current gold/s rising exponentially with time, one tenth of the exponential is applied as an increase to player action efficiency; dispel at 0 gold</t>
+    <t xml:space="preserve">Eats 10 gold/s rising exponentially with time, one tenth of the exponential is applied as an increase to player action efficiency; dispel at 0 gold</t>
   </si>
   <si>
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">Immediately when invoked, overrides other invocations in the room.
-Only disappears when dispelled.</t>
+    <t xml:space="preserve">Immediately when invoked, overrides other invocations in the room.</t>
   </si>
   <si>
     <t xml:space="preserve">Lamia</t>
@@ -7191,7 +7190,7 @@
         <v>0.015</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7208,14 +7207,14 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="34" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
@@ -7239,7 +7238,7 @@
         <v>0.025</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7250,7 +7249,7 @@
         <v>0.1</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7261,7 +7260,7 @@
         <v>0.3</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat(sim): Mercatus per-Sin signature clauses + wire the 0.5 player offline efficiency
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1045" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="708">
   <si>
     <t xml:space="preserve">Constant</t>
   </si>
@@ -1932,6 +1932,69 @@
   </si>
   <si>
     <t xml:space="preserve">Panvitium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-Sin signature clauses (slice 2 — §1.5 table as amended in session)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clause</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gulae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spendPerCapita ×1.25 for this trade (its revenue ×1.25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luxuriae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">its generation ×1.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avaritiae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">its depths 0.5% cheaper — invest cost ×0.995; refunds on the same basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tristitiae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+0.825% reprobate suicide-rate mul per depth (global)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Irae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+0.825% murder-rate mul per depth (global)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acediae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">revenue exempt from the ×0.5 offline efficiency; +0.825% offline gain rate mul per depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanagloriae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+0.25% of effective max influence as flat influence/s per full 10 depths (stepped)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superbiae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.25 / 1.33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depths ×1.25 dearer; its revenue ×1.33 and its generation ×1.33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Player base offline efficiency (Globals row 8, 0.5×) is now WIRED: resumeGame scales the catch-up by it; only Mercatus Acediae’s take is exempt.</t>
   </si>
   <si>
     <t xml:space="preserve">Vitium Compositum — multi-Sin toggles</t>
@@ -2419,7 +2482,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2612,7 +2675,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2620,11 +2691,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3162,46 +3229,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>632</v>
+        <v>653</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>633</v>
+        <v>654</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>634</v>
+        <v>655</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>635</v>
+        <v>656</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>636</v>
+        <v>657</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>637</v>
+        <v>658</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>638</v>
+        <v>659</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>639</v>
+        <v>660</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>640</v>
+        <v>661</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="53" t="s">
         <v>619</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>641</v>
+        <v>662</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>1</v>
@@ -3227,11 +3294,11 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="53" t="s">
         <v>620</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>642</v>
+        <v>663</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>1</v>
@@ -3257,11 +3324,11 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="53" t="s">
         <v>621</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>643</v>
+        <v>664</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>1</v>
@@ -3283,15 +3350,15 @@
         <v>0</v>
       </c>
       <c r="H7" s="45" t="s">
-        <v>644</v>
+        <v>665</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="53" t="s">
         <v>622</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>645</v>
+        <v>666</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>1</v>
@@ -3313,15 +3380,15 @@
         <v>0</v>
       </c>
       <c r="H8" s="45" t="s">
-        <v>646</v>
+        <v>667</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="53" t="s">
         <v>623</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>647</v>
+        <v>668</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>1</v>
@@ -3343,15 +3410,15 @@
         <v>0</v>
       </c>
       <c r="H9" s="45" t="s">
-        <v>648</v>
+        <v>669</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="53" t="s">
         <v>624</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>649</v>
+        <v>670</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>1</v>
@@ -3373,21 +3440,21 @@
         <v>0</v>
       </c>
       <c r="H10" s="45" t="s">
-        <v>650</v>
+        <v>671</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="53" t="s">
+      <c r="A11" s="54" t="s">
         <v>629</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>651</v>
+        <v>672</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>652</v>
+        <v>673</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0</v>
@@ -3396,18 +3463,18 @@
         <v>0</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>653</v>
+        <v>674</v>
       </c>
       <c r="H11" s="45" t="s">
         <v>516</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="54" t="s">
         <v>630</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>654</v>
+        <v>675</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>2</v>
@@ -3416,10 +3483,10 @@
         <v>0</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>655</v>
+        <v>676</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>656</v>
+        <v>677</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>0</v>
@@ -3429,20 +3496,20 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="54" t="s">
+      <c r="A13" s="55" t="s">
         <v>631</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>657</v>
+        <v>678</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>658</v>
+        <v>679</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>659</v>
+        <v>680</v>
       </c>
       <c r="F13" s="14" t="n">
         <f aca="false">0*Globals!$B$19</f>
@@ -3453,7 +3520,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="45" t="s">
-        <v>660</v>
+        <v>681</v>
       </c>
     </row>
     <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3487,26 +3554,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>661</v>
+        <v>682</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>662</v>
+        <v>683</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>663</v>
+        <v>684</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>664</v>
+        <v>685</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>665</v>
+        <v>686</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>666</v>
+        <v>687</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3520,7 +3587,7 @@
         <v>0.33</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>667</v>
+        <v>688</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3535,7 +3602,7 @@
         <v>0.33</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>668</v>
+        <v>689</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3550,7 +3617,7 @@
         <v>0.33</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>669</v>
+        <v>690</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3565,21 +3632,21 @@
         <v>0.33</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>670</v>
+        <v>691</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>671</v>
+        <v>692</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>672</v>
+        <v>693</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0.33</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>673</v>
+        <v>694</v>
       </c>
     </row>
   </sheetData>
@@ -3609,12 +3676,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>674</v>
+        <v>695</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>675</v>
+        <v>696</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3622,13 +3689,13 @@
         <v>326</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>676</v>
+        <v>697</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>677</v>
+        <v>698</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>678</v>
+        <v>699</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3636,7 +3703,7 @@
         <v>329</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>679</v>
+        <v>700</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>0</v>
@@ -3651,7 +3718,7 @@
         <v>331</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>680</v>
+        <v>701</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>0</v>
@@ -3666,7 +3733,7 @@
         <v>333</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>681</v>
+        <v>702</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>0</v>
@@ -3681,7 +3748,7 @@
         <v>335</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>682</v>
+        <v>703</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>0</v>
@@ -3696,7 +3763,7 @@
         <v>337</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>683</v>
+        <v>704</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>0</v>
@@ -3711,7 +3778,7 @@
         <v>339</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>684</v>
+        <v>705</v>
       </c>
       <c r="C10" s="14" t="n">
         <v>0</v>
@@ -3726,7 +3793,7 @@
         <v>341</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>685</v>
+        <v>706</v>
       </c>
       <c r="C11" s="14" t="n">
         <v>0</v>
@@ -3740,18 +3807,18 @@
       <c r="A12" s="9" t="s">
         <v>392</v>
       </c>
-      <c r="C12" s="55" t="n">
+      <c r="C12" s="56" t="n">
         <f aca="false">SUM(C5:C11)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="56" t="n">
+      <c r="D12" s="57" t="n">
         <f aca="false">SUM(D5:D11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>686</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>
@@ -8569,7 +8636,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="47.16"/>
@@ -8588,23 +8655,23 @@
         <v>586</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="48" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="49" t="s">
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="47" t="s">
         <v>588</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="48" t="s">
         <v>589</v>
       </c>
@@ -8615,7 +8682,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
         <v>591</v>
       </c>
@@ -8626,7 +8693,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
         <v>593</v>
       </c>
@@ -8634,7 +8701,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="48" t="s">
         <v>595</v>
       </c>
@@ -8645,7 +8712,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="48" t="s">
         <v>597</v>
       </c>
@@ -8656,7 +8723,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="48" t="s">
         <v>599</v>
       </c>
@@ -8667,11 +8734,11 @@
         <v>600</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
         <v>601</v>
       </c>
-      <c r="B11" s="50" t="n">
+      <c r="B11" s="49" t="n">
         <f aca="false">Globals!$B$14</f>
         <v>0.25</v>
       </c>
@@ -8679,7 +8746,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
         <v>603</v>
       </c>
@@ -8690,7 +8757,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
         <v>605</v>
       </c>
@@ -8701,7 +8768,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="48" t="s">
         <v>607</v>
       </c>
@@ -8710,7 +8777,7 @@
       </c>
       <c r="C14" s="48"/>
     </row>
-    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="48" t="s">
         <v>608</v>
       </c>
@@ -8721,7 +8788,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
         <v>610</v>
       </c>
@@ -8732,154 +8799,263 @@
         <v>611</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="49" t="s">
+    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="47" t="s">
         <v>612</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="48" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="48" t="s">
         <v>614</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="48" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="49" t="s">
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="47" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="49" t="s">
+    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="47" t="s">
         <v>617</v>
       </c>
-      <c r="B24" s="49" t="s">
+      <c r="B24" s="47" t="s">
         <v>618</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="48" t="s">
         <v>619</v>
       </c>
-      <c r="B25" s="51" t="b">
+      <c r="B25" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
         <v>620</v>
       </c>
-      <c r="B26" s="51" t="b">
+      <c r="B26" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="48" t="s">
         <v>621</v>
       </c>
-      <c r="B27" s="51" t="b">
+      <c r="B27" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
         <v>622</v>
       </c>
-      <c r="B28" s="51" t="b">
+      <c r="B28" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="48" t="s">
         <v>623</v>
       </c>
-      <c r="B29" s="51" t="b">
+      <c r="B29" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="s">
         <v>624</v>
       </c>
-      <c r="B30" s="51" t="b">
+      <c r="B30" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="48" t="s">
         <v>625</v>
       </c>
-      <c r="B31" s="51" t="b">
+      <c r="B31" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="48" t="s">
         <v>626</v>
       </c>
-      <c r="B32" s="51" t="b">
+      <c r="B32" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="48" t="s">
         <v>627</v>
       </c>
-      <c r="B33" s="51" t="b">
+      <c r="B33" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="48" t="s">
         <v>628</v>
       </c>
-      <c r="B34" s="51" t="b">
+      <c r="B34" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="48" t="s">
         <v>629</v>
       </c>
-      <c r="B35" s="51" t="b">
+      <c r="B35" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="48" t="s">
         <v>630</v>
       </c>
-      <c r="B36" s="51" t="b">
+      <c r="B36" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="48" t="s">
         <v>631</v>
       </c>
-      <c r="B37" s="51" t="b">
+      <c r="B37" s="50" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="51" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="51" t="s">
+        <v>633</v>
+      </c>
+      <c r="B40" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40" s="51" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="52" t="s">
+        <v>635</v>
+      </c>
+      <c r="B41" s="52" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C41" s="52" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="52" t="s">
+        <v>637</v>
+      </c>
+      <c r="B42" s="52" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C42" s="52" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="52" t="s">
+        <v>639</v>
+      </c>
+      <c r="B43" s="52" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="C43" s="52" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="52" t="s">
+        <v>641</v>
+      </c>
+      <c r="B44" s="52" t="n">
+        <v>0.00825</v>
+      </c>
+      <c r="C44" s="52" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="52" t="s">
+        <v>643</v>
+      </c>
+      <c r="B45" s="52" t="n">
+        <v>0.00825</v>
+      </c>
+      <c r="C45" s="52" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="52" t="s">
+        <v>645</v>
+      </c>
+      <c r="B46" s="52" t="n">
+        <v>0.00825</v>
+      </c>
+      <c r="C46" s="52" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="52" t="s">
+        <v>647</v>
+      </c>
+      <c r="B47" s="52" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="C47" s="52" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="52" t="s">
+        <v>649</v>
+      </c>
+      <c r="B48" s="52" t="s">
+        <v>650</v>
+      </c>
+      <c r="C48" s="52" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="52" t="s">
+        <v>652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(economy): retune slice 3 — VC canonical nine, Vegas/Crusade percentage semantics (ADR-027)
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="704">
   <si>
     <t xml:space="preserve">Constant</t>
   </si>
@@ -1911,18 +1911,6 @@
   </si>
   <si>
     <t xml:space="preserve">Doom gathering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loan Shark Op</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outrage Cycle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No-babies Movement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethnocentric Revolt</t>
   </si>
   <si>
     <t xml:space="preserve">Vegas</t>
@@ -3170,7 +3158,7 @@
       <c r="C21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
         <v>33</v>
       </c>
@@ -3212,35 +3200,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>656</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>657</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>658</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>659</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>661</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>327</v>
@@ -3251,7 +3239,7 @@
         <v>619</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>1</v>
@@ -3281,7 +3269,7 @@
         <v>620</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>1</v>
@@ -3311,7 +3299,7 @@
         <v>621</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>1</v>
@@ -3333,7 +3321,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="45" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3341,7 +3329,7 @@
         <v>622</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>1</v>
@@ -3363,7 +3351,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="45" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,7 +3359,7 @@
         <v>623</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>1</v>
@@ -3393,7 +3381,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="45" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3401,7 +3389,7 @@
         <v>624</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>1</v>
@@ -3423,21 +3411,21 @@
         <v>0</v>
       </c>
       <c r="H10" s="45" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="52" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>0</v>
@@ -3446,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="H11" s="45" t="s">
         <v>516</v>
@@ -3454,10 +3442,10 @@
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="52" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>2</v>
@@ -3466,10 +3454,10 @@
         <v>0</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="G12" s="13" t="n">
         <v>0</v>
@@ -3480,19 +3468,19 @@
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="53" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">0*Globals!$B$19</f>
@@ -3503,7 +3491,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="45" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
     </row>
     <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3537,26 +3525,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3570,7 +3558,7 @@
         <v>0.33</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,7 +3573,7 @@
         <v>0.33</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3600,7 +3588,7 @@
         <v>0.33</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3615,21 +3603,21 @@
         <v>0.33</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>0.33</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
     </row>
   </sheetData>
@@ -3659,12 +3647,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3672,13 +3660,13 @@
         <v>325</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3686,7 +3674,7 @@
         <v>328</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>0</v>
@@ -3701,7 +3689,7 @@
         <v>330</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>0</v>
@@ -3716,7 +3704,7 @@
         <v>332</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>0</v>
@@ -3731,7 +3719,7 @@
         <v>334</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>0</v>
@@ -3746,7 +3734,7 @@
         <v>336</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>0</v>
@@ -3761,7 +3749,7 @@
         <v>338</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>0</v>
@@ -3776,7 +3764,7 @@
         <v>340</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>0</v>
@@ -3801,7 +3789,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>
@@ -8896,151 +8884,120 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="48" t="s">
+    <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="47" t="s">
         <v>628</v>
       </c>
-      <c r="B34" s="50" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="48" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="47" t="s">
         <v>629</v>
       </c>
-      <c r="B35" s="50" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="48" t="s">
+      <c r="B36" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C36" s="47" t="s">
         <v>630</v>
-      </c>
-      <c r="B36" s="50" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="48" t="s">
         <v>631</v>
       </c>
-      <c r="B37" s="50" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="B37" s="48" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C37" s="48" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="48" t="s">
+        <v>633</v>
+      </c>
+      <c r="B38" s="48" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C38" s="48" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="47" t="s">
-        <v>632</v>
+      <c r="A39" s="48" t="s">
+        <v>635</v>
+      </c>
+      <c r="B39" s="48" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="C39" s="48" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="47" t="s">
-        <v>633</v>
-      </c>
-      <c r="B40" s="47" t="s">
-        <v>0</v>
-      </c>
-      <c r="C40" s="47" t="s">
-        <v>634</v>
+      <c r="A40" s="48" t="s">
+        <v>637</v>
+      </c>
+      <c r="B40" s="48" t="n">
+        <v>0.00825</v>
+      </c>
+      <c r="C40" s="48" t="s">
+        <v>638</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="48" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="B41" s="48" t="n">
-        <v>1.25</v>
+        <v>0.00825</v>
       </c>
       <c r="C41" s="48" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="48" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="B42" s="48" t="n">
-        <v>1.25</v>
+        <v>0.00825</v>
       </c>
       <c r="C42" s="48" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="48" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B43" s="48" t="n">
-        <v>0.995</v>
+        <v>0.0025</v>
       </c>
       <c r="C43" s="48" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="48" t="s">
-        <v>641</v>
-      </c>
-      <c r="B44" s="48" t="n">
-        <v>0.00825</v>
+        <v>645</v>
+      </c>
+      <c r="B44" s="48" t="s">
+        <v>646</v>
       </c>
       <c r="C44" s="48" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="48" t="s">
-        <v>643</v>
-      </c>
-      <c r="B45" s="48" t="n">
-        <v>0.00825</v>
-      </c>
-      <c r="C45" s="48" t="s">
-        <v>644</v>
-      </c>
-    </row>
+        <v>647</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="48" t="s">
-        <v>645</v>
-      </c>
-      <c r="B46" s="48" t="n">
-        <v>0.00825</v>
-      </c>
-      <c r="C46" s="48" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="48" t="s">
-        <v>647</v>
-      </c>
-      <c r="B47" s="48" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="C47" s="48" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="48" t="s">
-        <v>649</v>
-      </c>
-      <c r="B48" s="48" t="s">
-        <v>650</v>
-      </c>
-      <c r="C48" s="48" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="48" t="s">
-        <v>652</v>
-      </c>
-    </row>
+    <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
feat(economy): retune slice 5 — the 72-sigil respecification (ADR-029)
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -4194,15 +4194,15 @@
         <v>106</v>
       </c>
       <c r="F5" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H5" s="18" t="n">
         <f aca="false">IF(F5="","",F5*IF(E5="linear",G5,IF(E5="log",LN(G5+1),SQRT(G5))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4222,15 +4222,15 @@
         <v>106</v>
       </c>
       <c r="F6" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H6" s="18" t="n">
         <f aca="false">IF(F6="","",F6*IF(E6="linear",G6,IF(E6="log",LN(G6+1),SQRT(G6))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4250,15 +4250,15 @@
         <v>106</v>
       </c>
       <c r="F7" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>100000</v>
       </c>
       <c r="H7" s="18" t="n">
         <f aca="false">IF(F7="","",F7*IF(E7="linear",G7,IF(E7="log",LN(G7+1),SQRT(G7))))</f>
-        <v>0</v>
+        <v>0.0316227766016838</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4278,15 +4278,15 @@
         <v>106</v>
       </c>
       <c r="F8" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>10000</v>
       </c>
       <c r="H8" s="18" t="n">
         <f aca="false">IF(F8="","",F8*IF(E8="linear",G8,IF(E8="log",LN(G8+1),SQRT(G8))))</f>
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4306,15 +4306,15 @@
         <v>106</v>
       </c>
       <c r="F9" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>100000</v>
       </c>
       <c r="H9" s="18" t="n">
         <f aca="false">IF(F9="","",F9*IF(E9="linear",G9,IF(E9="log",LN(G9+1),SQRT(G9))))</f>
-        <v>0</v>
+        <v>0.0316227766016838</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4334,15 +4334,15 @@
         <v>106</v>
       </c>
       <c r="F10" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H10" s="18" t="n">
         <f aca="false">IF(F10="","",F10*IF(E10="linear",G10,IF(E10="log",LN(G10+1),SQRT(G10))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4362,15 +4362,15 @@
         <v>106</v>
       </c>
       <c r="F11" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H11" s="18" t="n">
         <f aca="false">IF(F11="","",F11*IF(E11="linear",G11,IF(E11="log",LN(G11+1),SQRT(G11))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4390,15 +4390,15 @@
         <v>106</v>
       </c>
       <c r="F12" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H12" s="18" t="n">
         <f aca="false">IF(F12="","",F12*IF(E12="linear",G12,IF(E12="log",LN(G12+1),SQRT(G12))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4418,15 +4418,15 @@
         <v>106</v>
       </c>
       <c r="F13" s="17" t="n">
-        <f aca="false">0.00005*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.00005*Globals!$B$21</f>
+        <v>5E-005</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H13" s="18" t="n">
         <f aca="false">IF(F13="","",F13*IF(E13="linear",G13,IF(E13="log",LN(G13+1),SQRT(G13))))</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4446,15 +4446,15 @@
         <v>106</v>
       </c>
       <c r="F14" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H14" s="18" t="n">
         <f aca="false">IF(F14="","",F14*IF(E14="linear",G14,IF(E14="log",LN(G14+1),SQRT(G14))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4474,15 +4474,15 @@
         <v>106</v>
       </c>
       <c r="F15" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H15" s="18" t="n">
         <f aca="false">IF(F15="","",F15*IF(E15="linear",G15,IF(E15="log",LN(G15+1),SQRT(G15))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4502,15 +4502,15 @@
         <v>106</v>
       </c>
       <c r="F16" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>100000</v>
       </c>
       <c r="H16" s="18" t="n">
         <f aca="false">IF(F16="","",F16*IF(E16="linear",G16,IF(E16="log",LN(G16+1),SQRT(G16))))</f>
-        <v>0</v>
+        <v>0.0316227766016838</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4530,15 +4530,15 @@
         <v>106</v>
       </c>
       <c r="F17" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H17" s="18" t="n">
         <f aca="false">IF(F17="","",F17*IF(E17="linear",G17,IF(E17="log",LN(G17+1),SQRT(G17))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4558,15 +4558,15 @@
         <v>106</v>
       </c>
       <c r="F18" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H18" s="18" t="n">
         <f aca="false">IF(F18="","",F18*IF(E18="linear",G18,IF(E18="log",LN(G18+1),SQRT(G18))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4586,15 +4586,15 @@
         <v>106</v>
       </c>
       <c r="F19" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H19" s="18" t="n">
         <f aca="false">IF(F19="","",F19*IF(E19="linear",G19,IF(E19="log",LN(G19+1),SQRT(G19))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4614,15 +4614,15 @@
         <v>106</v>
       </c>
       <c r="F20" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G20" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H20" s="18" t="n">
         <f aca="false">IF(F20="","",F20*IF(E20="linear",G20,IF(E20="log",LN(G20+1),SQRT(G20))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4642,15 +4642,15 @@
         <v>106</v>
       </c>
       <c r="F21" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H21" s="18" t="n">
         <f aca="false">IF(F21="","",F21*IF(E21="linear",G21,IF(E21="log",LN(G21+1),SQRT(G21))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4670,15 +4670,15 @@
         <v>106</v>
       </c>
       <c r="F22" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H22" s="18" t="n">
         <f aca="false">IF(F22="","",F22*IF(E22="linear",G22,IF(E22="log",LN(G22+1),SQRT(G22))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4698,15 +4698,15 @@
         <v>106</v>
       </c>
       <c r="F23" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H23" s="18" t="n">
         <f aca="false">IF(F23="","",F23*IF(E23="linear",G23,IF(E23="log",LN(G23+1),SQRT(G23))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4753,15 +4753,15 @@
         <v>106</v>
       </c>
       <c r="F25" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H25" s="18" t="n">
         <f aca="false">IF(F25="","",F25*IF(E25="linear",G25,IF(E25="log",LN(G25+1),SQRT(G25))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4781,15 +4781,15 @@
         <v>106</v>
       </c>
       <c r="F26" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G26" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H26" s="18" t="n">
         <f aca="false">IF(F26="","",F26*IF(E26="linear",G26,IF(E26="log",LN(G26+1),SQRT(G26))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4809,15 +4809,15 @@
         <v>106</v>
       </c>
       <c r="F27" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H27" s="18" t="n">
         <f aca="false">IF(F27="","",F27*IF(E27="linear",G27,IF(E27="log",LN(G27+1),SQRT(G27))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4837,15 +4837,15 @@
         <v>106</v>
       </c>
       <c r="F28" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H28" s="18" t="n">
         <f aca="false">IF(F28="","",F28*IF(E28="linear",G28,IF(E28="log",LN(G28+1),SQRT(G28))))</f>
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4892,15 +4892,15 @@
         <v>106</v>
       </c>
       <c r="F30" s="17" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>1000</v>
       </c>
       <c r="H30" s="18" t="n">
         <f aca="false">IF(F30="","",F30*IF(E30="linear",G30,IF(E30="log",LN(G30+1),SQRT(G30))))</f>
-        <v>0</v>
+        <v>0.00316227766016838</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5001,15 +5001,15 @@
         <v>164</v>
       </c>
       <c r="F34" s="30" t="n">
-        <f aca="false">0.5*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.5*Globals!$B$21</f>
+        <v>0.5</v>
       </c>
       <c r="G34" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H34" s="5" t="n">
         <f aca="false">IF(F34="","",F34*IF(E34="linear",G34,IF(E34="log",LN(G34+1),SQRT(G34))))</f>
-        <v>0</v>
+        <v>9.21034037697618</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5056,15 +5056,15 @@
         <v>164</v>
       </c>
       <c r="F36" s="31" t="n">
-        <f aca="false">0.01*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.01*Globals!$B$21</f>
+        <v>0.01</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>5832000</v>
       </c>
       <c r="H36" s="18" t="n">
         <f aca="false">IF(F36="","",F36*IF(E36="linear",G36,IF(E36="log",LN(G36+1),SQRT(G36))))</f>
-        <v>0</v>
+        <v>0.155788707241384</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5084,15 +5084,15 @@
         <v>164</v>
       </c>
       <c r="F37" s="31" t="n">
-        <f aca="false">0.01*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.01*Globals!$B$21</f>
+        <v>0.01</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H37" s="18" t="n">
         <f aca="false">IF(F37="","",F37*IF(E37="linear",G37,IF(E37="log",LN(G37+1),SQRT(G37))))</f>
-        <v>0</v>
+        <v>0.184206807539524</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5490,15 +5490,15 @@
         <v>164</v>
       </c>
       <c r="F52" s="30" t="n">
-        <f aca="false">3*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">3*Globals!$B$21</f>
+        <v>3</v>
       </c>
       <c r="G52" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H52" s="5" t="n">
         <f aca="false">IF(F52="","",F52*IF(E52="linear",G52,IF(E52="log",LN(G52+1),SQRT(G52))))</f>
-        <v>0</v>
+        <v>55.2620422618571</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5734,15 +5734,15 @@
         <v>164</v>
       </c>
       <c r="F61" s="30" t="n">
-        <f aca="false">0.3*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.3*Globals!$B$21</f>
+        <v>0.3</v>
       </c>
       <c r="G61" s="4" t="n">
         <v>100</v>
       </c>
       <c r="H61" s="5" t="n">
         <f aca="false">IF(F61="","",F61*IF(E61="linear",G61,IF(E61="log",LN(G61+1),SQRT(G61))))</f>
-        <v>0</v>
+        <v>1.38453615505238</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5951,15 +5951,15 @@
         <v>106</v>
       </c>
       <c r="F69" s="31" t="n">
-        <f aca="false">0.0001*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.0001*Globals!$B$21</f>
+        <v>0.0001</v>
       </c>
       <c r="G69" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H69" s="18" t="n">
         <f aca="false">IF(F69="","",F69*IF(E69="linear",G69,IF(E69="log",LN(G69+1),SQRT(G69))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6060,15 +6060,15 @@
         <v>164</v>
       </c>
       <c r="F73" s="30" t="n">
-        <f aca="false">0.5*Globals!$B$22</f>
-        <v>0</v>
+        <f aca="false">0.5*Globals!$B$21</f>
+        <v>0.5</v>
       </c>
       <c r="G73" s="4" t="n">
         <v>100000000</v>
       </c>
       <c r="H73" s="5" t="n">
         <f aca="false">IF(F73="","",F73*IF(E73="linear",G73,IF(E73="log",LN(G73+1),SQRT(G73))))</f>
-        <v>0</v>
+        <v>9.21034037697618</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8912,7 +8912,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="48" t="s">
         <v>633</v>
       </c>

</xml_diff>